<commit_message>
WIP TRS02. (Completed write FRU, WIP read FRU)
</commit_message>
<xml_diff>
--- a/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/FRU Array.xlsx
+++ b/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/FRU Array.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Emerson\SolaHD\SDU-DC-UPS-EIP\PCBA\TesterSpecific\FRU PROGRAMMING TOOLKIT\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{EA45878D-3E51-48B3-9E78-E57D4D0819C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{308A4A56-7819-444D-B8C5-080C05EED5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9538C7C6-F33D-4746-B93C-9BE93615E927}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{9538C7C6-F33D-4746-B93C-9BE93615E927}"/>
   </bookViews>
   <sheets>
     <sheet name="FRU Array" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
   <si>
     <t>FRU Information</t>
   </si>
@@ -244,7 +244,13 @@
     <t>0624</t>
   </si>
   <si>
+    <t>02C0</t>
+  </si>
+  <si>
     <t>0600</t>
+  </si>
+  <si>
+    <t>FF</t>
   </si>
 </sst>
 </file>
@@ -1573,7 +1579,7 @@
         <v>36</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C32" s="2">
         <v>0</v>
@@ -1627,6 +1633,12 @@
     <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>40</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="D36">
         <v>128</v>

</xml_diff>

<commit_message>
Added STLink Software & STLink in Teststand
</commit_message>
<xml_diff>
--- a/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/FRU Array.xlsx
+++ b/PCBA/TesterSpecific/FRU PROGRAMMING TOOLKIT/Data/FRU Array.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Emerson\SolaHD\SDU-DC-UPS-EIP\PCBA\TesterSpecific\FRU PROGRAMMING TOOLKIT\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{308A4A56-7819-444D-B8C5-080C05EED5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D3BE0B03-20FE-4720-96FB-43A6447BBFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{9538C7C6-F33D-4746-B93C-9BE93615E927}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>FRU Information</t>
   </si>
@@ -142,9 +142,6 @@
     <t>Flyback TRF Temp C.C 1</t>
   </si>
   <si>
-    <t>Event Data</t>
-  </si>
-  <si>
     <t>0022</t>
   </si>
   <si>
@@ -251,6 +248,12 @@
   </si>
   <si>
     <t>FF</t>
+  </si>
+  <si>
+    <t>=B36+0008</t>
+  </si>
+  <si>
+    <t>Event Data 1</t>
   </si>
 </sst>
 </file>
@@ -1215,10 +1218,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="D6">
         <v>128</v>
@@ -1229,10 +1232,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="D7">
         <v>32</v>
@@ -1243,10 +1246,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D8">
         <v>32</v>
@@ -1257,10 +1260,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D9">
         <v>128</v>
@@ -1271,7 +1274,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="2">
         <v>4141</v>
@@ -1285,10 +1288,10 @@
         <v>15</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="D11">
         <v>128</v>
@@ -1299,10 +1302,10 @@
         <v>16</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12">
         <v>128</v>
@@ -1327,7 +1330,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C14" s="2">
         <v>0</v>
@@ -1341,7 +1344,7 @@
         <v>19</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C15" s="2">
         <v>32</v>
@@ -1355,7 +1358,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2">
         <v>14</v>
@@ -1369,7 +1372,7 @@
         <v>21</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C17" s="2">
         <v>78</v>
@@ -1383,10 +1386,10 @@
         <v>22</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D18">
         <v>128</v>
@@ -1397,10 +1400,10 @@
         <v>23</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D19">
         <v>128</v>
@@ -1411,7 +1414,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C20" s="2">
         <v>0</v>
@@ -1425,7 +1428,7 @@
         <v>25</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2">
         <v>0</v>
@@ -1439,7 +1442,7 @@
         <v>26</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C22" s="2">
         <v>0</v>
@@ -1453,7 +1456,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C23" s="2">
         <v>0</v>
@@ -1467,7 +1470,7 @@
         <v>28</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2">
         <v>0</v>
@@ -1481,7 +1484,7 @@
         <v>29</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C25" s="2">
         <v>0</v>
@@ -1495,7 +1498,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C26" s="2">
         <v>0</v>
@@ -1509,7 +1512,7 @@
         <v>31</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C27" s="2">
         <v>0</v>
@@ -1523,7 +1526,7 @@
         <v>32</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2">
         <v>0</v>
@@ -1537,7 +1540,7 @@
         <v>33</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C29" s="2">
         <v>0</v>
@@ -1551,7 +1554,7 @@
         <v>34</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C30" s="2">
         <v>0</v>
@@ -1565,7 +1568,7 @@
         <v>35</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C31" s="2">
         <v>0</v>
@@ -1579,7 +1582,7 @@
         <v>36</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C32" s="2">
         <v>0</v>
@@ -1593,7 +1596,7 @@
         <v>37</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" s="2">
         <v>0</v>
@@ -1607,7 +1610,7 @@
         <v>38</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C34" s="2">
         <v>0</v>
@@ -1621,7 +1624,7 @@
         <v>39</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C35" s="2">
         <v>0</v>
@@ -1632,16 +1635,21 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="B37" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="D36">
-        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:4">

</xml_diff>